<commit_message>
Rework Felpudos Cotizador: material always selectable, add logo complexity
Per user feedback: marca/espesor now drives base cost regardless of
whether the mat has a logo (previously con-logo pricing was locked to
Confort Mat only). Adds an independent "complejidad de logo"
(Simple/Media/Compleja) factor with its own multipliers on material and
labor cost. Only "Media" is calibrated against real data (the 4
handwritten examples); Simple/Compleja multipliers are flagged as
estimates pending real reference quotes.
</commit_message>
<xml_diff>
--- a/contexto-marcas/felpudos-y-servicios/herramientas/Felpudos_Cotizador.xlsx
+++ b/contexto-marcas/felpudos-y-servicios/herramientas/Felpudos_Cotizador.xlsx
@@ -18,11 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="&quot;S/&quot; #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="166" formatCode="&quot;S/&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,8 +62,15 @@
       <name val="Arial"/>
       <color rgb="000000FF"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00CC0000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +90,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
     <fill>
@@ -116,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -135,7 +148,16 @@
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -147,10 +169,13 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -524,15 +549,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -545,523 +571,611 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Transcrito de notas de costeo manuscritas (fotos compartidas 2026-07-21). Celdas en amarillo/azul = valores base que alimentan las fórmulas del Cotizador. Ver supuestos y alertas en la pestaña 'Notas y Supuestos'.</t>
+          <t>Transcrito de notas de costeo manuscritas (fotos 2026-07-21). Celdas amarillas = datos reales confirmados. Celdas ámbar = estimaciones a validar (ver columna Nota). El Cotizador usa estos valores — cambia algo aquí y se actualiza todo solo.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1. FELPUDO DE VINILO CON LOGO (personalizado, marca base Confort Mat)</t>
+          <t>1. FELPUDO DE VINILO — MATERIALES BASE (aplica con o sin logo)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Concepto</t>
+          <t>Marca</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Valor</t>
+          <t>Espesor</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Costo (S//m²)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Margen sugerido</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Clave (marca+espesor)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Costo material base</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
+          <t>Confort Mat</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>14-15mm</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
         <v>59.17</v>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>S//m²</t>
+      <c r="D6" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Confort Mat 14-15mm</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Usado en los 3 ejemplos reales con logo (Vet. Orbegoso, FINA, Bar Popular)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Costo material extra (ribete de recorte)</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>94.90000000000001</v>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>S//m</t>
+          <t>Multilop</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>12mm</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>79.08</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Multilop 12mm</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Convertido de S/94.90/m lineal ÷ 1.20m de ancho de rollo</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Longitud extra si área &lt; 1.00 m²</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>m</t>
+          <t>Multilop</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>15mm</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>105.75</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Multilop 15mm</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Convertido de S/126.90/m lineal ÷ 1.20m</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Longitud extra si área ≥ 1.00 m²</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>m</t>
+          <t>Paolo</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>12mm</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Paolo 12mm</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Convertido de S/50.00/m lineal ÷ 1.20m</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Mano de obra — componente fijo</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>80</v>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>S/</t>
+          <t>Paolo</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>15mm</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>79.17</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Paolo 15mm</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Convertido de S/95.00/m lineal ÷ 1.20m (ver Notas: discrepancia S/90 vs S/95 en el original)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Mano de obra — componente variable</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>37.04</v>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>S//m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Ajuste fijo de acabado (tapiz)</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>S/</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Margen sugerido</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n">
+          <t>Q Rubber</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>13-14mm</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>59.17</v>
+      </c>
+      <c r="D11" s="7" t="n">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>2. FELPUDO DE VINILO EN ROLLO (sin logo) — ancho fijo de rollo 1.20 m</t>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Q Rubber 13-14mm</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Convertido de S/71.00/m lineal ÷ 1.20m</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>1b. FELPUDO DE VINILO — NIVELES DE COMPLEJIDAD DEL LOGO (solo si lleva logo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Nivel</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Mult. costo material extra</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Mult. mano de obra</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>ESTIMADO — sin datos reales. Ajustar cuando haya ejemplos (1-2 colores, texto simple).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Baseline = los 4 ejemplos reales que sí tenemos (logos con 2-3 colores, tipo Vet.Orbegoso/FINA/Bar Popular).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Espesor</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Costo (S//m)</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Margen sugerido</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Precio venta (S//m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Multilop</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>12mm</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>94.90000000000001</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E18" s="8">
-        <f>ROUND(C18/(1-D18),2)</f>
-        <v/>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>Multilop 12mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Multilop</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>15mm</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>126.9</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E19" s="8">
-        <f>ROUND(C19/(1-D19),2)</f>
-        <v/>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>Multilop 15mm</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Compleja</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>ESTIMADO — sin datos reales. Ajustar cuando haya ejemplos (4+ colores, degradados, detalle fino).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>1c. FELPUDO DE VINILO — OTROS COSTOS DEL LOGO (nivel 'Media', antes de multiplicador)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Paolo</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>12mm</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E20" s="8">
-        <f>ROUND(C20/(1-D20),2)</f>
-        <v/>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>Paolo 12mm</t>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Paolo</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>15mm</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>95</v>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E21" s="8">
-        <f>ROUND(C21/(1-D21),2)</f>
-        <v/>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>Paolo 15mm</t>
+          <t>Costo material extra ribete (por m lineal)</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>S//m</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Q Rubber</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>13-14mm</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>71</v>
-      </c>
-      <c r="D22" s="7" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E22" s="8">
-        <f>ROUND(C22/(1-D22),2)</f>
-        <v/>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Q Rubber 13-14mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>3. FELPUDOS MIXTOS (retienen polvo y secan, perfil de jebe — marca base Confort Mat)</t>
+          <t>Longitud extra si área &lt; 1.00 m²</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Longitud extra si área ≥ 1.00 m²</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Mano de obra — componente fijo</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>S/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Mano de obra — componente variable</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>37.04</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>S//m²</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Ajuste fijo de acabado (tapiz)</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>S/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>2. FELPUDOS MIXTOS (retienen polvo y secan, perfil de jebe — marca base Confort Mat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Unidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Costo material</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>S//m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Costo perfil (ribete de jebe)</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>S//m</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Extra fijo sobre perímetro</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>m</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Mano de obra — componente fijo</t>
+          <t>Costo material</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>S/</t>
+          <t>S//m²</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Mano de obra — componente variable</t>
+          <t>Costo perfil (ribete de jebe)</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>16.67</v>
+        <v>9</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>S//m²</t>
+          <t>S//m</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>Extra fijo sobre perímetro</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Mano de obra — componente fijo</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>S/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Mano de obra — componente variable</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>S//m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
           <t>Margen sugerido</t>
         </is>
       </c>
-      <c r="B32" s="7" t="n">
+      <c r="B35" s="7" t="n">
         <v>0.33</v>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>4. PISO ANTIFATIGA</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>3. PISO ANTIFATIGA</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>Espesor</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Costo (S//m²)</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>Margen sugerido</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Precio ref. (1.50×0.90m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Clave</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>Paolo</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>9mm</t>
         </is>
       </c>
-      <c r="C37" s="6" t="n">
+      <c r="C39" s="6" t="n">
         <v>37.04</v>
       </c>
-      <c r="D37" s="7" t="n">
+      <c r="D39" s="7" t="n">
         <v>0.58</v>
       </c>
-      <c r="E37" s="8">
-        <f>ROUND(C37*1.35/(1-D37),2)</f>
-        <v/>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>Paolo 9mm</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>Q Rubber</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>13mm</t>
         </is>
       </c>
-      <c r="C38" s="6" t="n">
+      <c r="C40" s="6" t="n">
         <v>87.41</v>
       </c>
-      <c r="D38" s="7" t="n">
+      <c r="D40" s="7" t="n">
         <v>0.41</v>
       </c>
-      <c r="E38" s="8">
-        <f>ROUND(C38*1.35/(1-D38),2)</f>
-        <v/>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t>Q Rubber 13mm</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1073,10 +1187,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -1094,14 +1208,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Llena solo las celdas amarillas. El precio sugerido se calcula automáticamente a partir de los datos de costeo de la pestaña 'Datos Base'. Revisa 'Notas y Supuestos' antes de usarlo para cotizar en firme.</t>
+          <t>Llena solo las celdas amarillas. Las celdas ámbar en 'Datos Base' (niveles de complejidad Simple/Compleja) son estimaciones — ajústalas ahí cuando tengas datos reales.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>A. FELPUDO DE VINILO (personalizado con logo, o en rollo sin logo)</t>
+          <t>A. FELPUDO DE VINILO (con o sin logo)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1225,7 @@
           <t>Ancho (m)</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="12" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -1121,370 +1235,396 @@
           <t>Alto / largo (m)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="12" t="n">
         <v>0.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>¿Lleva logo?</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Sí</t>
+          <t>Marca y espesor de la base</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Confort Mat 14-15mm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Si NO lleva logo — Marca y espesor del rollo</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Multilop 12mm</t>
+          <t>¿Lleva logo?</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>Complejidad del logo (solo si lleva logo)</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
           <t>Margen deseado (%) — vacío = usar el sugerido</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="B10" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>RESULTADOS</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Área (m²)</t>
-        </is>
-      </c>
-      <c r="B12" s="11">
-        <f>B5*B6</f>
-        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Costo materiales (S/)</t>
-        </is>
-      </c>
-      <c r="B13" s="8">
-        <f>IF(B7="Sí", B12*'Datos Base'!$B$6 + IF(B12&lt;1,'Datos Base'!$B$8,'Datos Base'!$B$9)*'Datos Base'!$B$7, B6*INDEX('Datos Base'!$C$18:$C$22,MATCH(B8,'Datos Base'!$F$18:$F$22,0)))</f>
+          <t>Área (m²)</t>
+        </is>
+      </c>
+      <c r="B13" s="14">
+        <f>B5*B6</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Costo mano de obra (S/)</t>
-        </is>
-      </c>
-      <c r="B14" s="8">
-        <f>IF(B7="Sí", 'Datos Base'!$B$10 + 'Datos Base'!$B$11*B12, 0)</f>
+          <t>Costo material base (S/)</t>
+        </is>
+      </c>
+      <c r="B14" s="15">
+        <f>B13*INDEX('Datos Base'!$C$6:$C$11,MATCH(B7,'Datos Base'!$F$6:$F$11,0))</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Costo total (S/)</t>
-        </is>
-      </c>
-      <c r="B15" s="8">
-        <f>B13+B14</f>
+          <t>Costo material extra por logo (S/)</t>
+        </is>
+      </c>
+      <c r="B15" s="15">
+        <f>IF(B8="Sí", IF(B13&lt;1,'Datos Base'!$B$22,'Datos Base'!$B$23)*'Datos Base'!$B$21*INDEX('Datos Base'!$B$15:$B$17,MATCH(B9,'Datos Base'!$A$15:$A$17,0)), 0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Margen aplicado (%)</t>
-        </is>
-      </c>
-      <c r="B16" s="12">
-        <f>IF(B9&lt;&gt;"", B9, IF(B7="Sí", 'Datos Base'!$B$13, INDEX('Datos Base'!$D$18:$D$22,MATCH(B8,'Datos Base'!$F$18:$F$22,0))))</f>
+          <t>Costo mano de obra (S/)</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>IF(B8="Sí", ('Datos Base'!$B$24+'Datos Base'!$B$25*B13)*INDEX('Datos Base'!$C$15:$C$17,MATCH(B9,'Datos Base'!$A$15:$A$17,0)), 0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>Costo total (S/)</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>B14+B15+B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Margen aplicado (%)</t>
+        </is>
+      </c>
+      <c r="B18" s="16">
+        <f>IF(B10&lt;&gt;"", B10, INDEX('Datos Base'!$D$6:$D$11,MATCH(B7,'Datos Base'!$F$6:$F$11,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
           <t>Ajuste fijo de acabado (S/, solo con logo)</t>
         </is>
       </c>
-      <c r="B17" s="8">
-        <f>IF(B7="Sí",'Datos Base'!$B$12,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="B19" s="15">
+        <f>IF(B8="Sí",'Datos Base'!$B$26,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>PRECIO SUGERIDO (S/)</t>
         </is>
       </c>
-      <c r="B18" s="13">
-        <f>ROUND(B15/(1-B16)+B17,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="B20" s="17">
+        <f>ROUND(B17/(1-B18)+B19,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>B. FELPUDOS MIXTOS</t>
         </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Ancho (m)</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Alto / largo (m)</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
+          <t>Ancho (m)</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Alto / largo (m)</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t>Margen deseado (%) — vacío = usar el sugerido</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="B26" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>RESULTADOS</t>
         </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Área (m²)</t>
-        </is>
-      </c>
-      <c r="B27" s="11">
-        <f>B22*B23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Perímetro + extra (m)</t>
-        </is>
-      </c>
-      <c r="B28" s="11">
-        <f>2*(B22+B23)+'Datos Base'!$B$29</f>
-        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Costo materiales (S/)</t>
-        </is>
-      </c>
-      <c r="B29" s="8">
-        <f>B27*'Datos Base'!$B$27+B28*'Datos Base'!$B$28</f>
+          <t>Área (m²)</t>
+        </is>
+      </c>
+      <c r="B29" s="14">
+        <f>B24*B25</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Costo mano de obra (S/)</t>
-        </is>
-      </c>
-      <c r="B30" s="8">
-        <f>'Datos Base'!$B$30+'Datos Base'!$B$31*B27</f>
+          <t>Perímetro + extra (m)</t>
+        </is>
+      </c>
+      <c r="B30" s="14">
+        <f>2*(B24+B25)+'Datos Base'!$B$32</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Costo total (S/)</t>
-        </is>
-      </c>
-      <c r="B31" s="8">
-        <f>B29+B30</f>
+          <t>Costo materiales (S/)</t>
+        </is>
+      </c>
+      <c r="B31" s="15">
+        <f>B29*'Datos Base'!$B$30+B30*'Datos Base'!$B$31</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>Costo mano de obra (S/)</t>
+        </is>
+      </c>
+      <c r="B32" s="15">
+        <f>'Datos Base'!$B$33+'Datos Base'!$B$34*B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Costo total (S/)</t>
+        </is>
+      </c>
+      <c r="B33" s="15">
+        <f>B31+B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
           <t>Margen aplicado (%)</t>
         </is>
       </c>
-      <c r="B32" s="12">
-        <f>IF(B24&lt;&gt;"",B24,'Datos Base'!$B$32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="B34" s="16">
+        <f>IF(B26&lt;&gt;"",B26,'Datos Base'!$B$35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>PRECIO SUGERIDO (S/)</t>
         </is>
       </c>
-      <c r="B33" s="13">
-        <f>ROUND(B31/(1-B32),2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="B35" s="17">
+        <f>ROUND(B33/(1-B34),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>C. PISO ANTIFATIGA</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Ancho (m)</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>Alto / largo (m)</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="n">
-        <v>0.9</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Marca y espesor</t>
-        </is>
-      </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>Paolo 9mm</t>
-        </is>
+          <t>Ancho (m)</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
+          <t>Alto / largo (m)</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Marca y espesor</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>Paolo 9mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
           <t>Margen deseado (%) — vacío = usar el sugerido</t>
         </is>
       </c>
-      <c r="B40" s="7" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="B42" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>RESULTADOS</t>
         </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Área (m²)</t>
-        </is>
-      </c>
-      <c r="B43" s="11">
-        <f>B37*B38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Costo por m² (S/)</t>
-        </is>
-      </c>
-      <c r="B44" s="8">
-        <f>INDEX('Datos Base'!$C$37:$C$38,MATCH(B39,'Datos Base'!$F$37:$F$38,0))</f>
-        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Costo total (S/)</t>
-        </is>
-      </c>
-      <c r="B45" s="8">
-        <f>B43*B44</f>
+          <t>Área (m²)</t>
+        </is>
+      </c>
+      <c r="B45" s="14">
+        <f>B39*B40</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
+          <t>Costo por m² (S/)</t>
+        </is>
+      </c>
+      <c r="B46" s="15">
+        <f>INDEX('Datos Base'!$C$39:$C$40,MATCH(B41,'Datos Base'!$F$39:$F$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Costo total (S/)</t>
+        </is>
+      </c>
+      <c r="B47" s="15">
+        <f>B45*B46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
           <t>Margen aplicado (%)</t>
         </is>
       </c>
-      <c r="B46" s="12">
-        <f>IF(B40&lt;&gt;"",B40,INDEX('Datos Base'!$D$37:$D$38,MATCH(B39,'Datos Base'!$F$37:$F$38,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="B48" s="16">
+        <f>IF(B42&lt;&gt;"",B42,INDEX('Datos Base'!$D$39:$D$40,MATCH(B41,'Datos Base'!$F$39:$F$40,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>PRECIO SUGERIDO (S/)</t>
         </is>
       </c>
-      <c r="B47" s="13">
-        <f>ROUND(B45/(1-B46),2)</f>
+      <c r="B49" s="17">
+        <f>ROUND(B47/(1-B48),2)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A4:E4"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A4:F4"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Confort Mat 14-15mm,Multilop 12mm,Multilop 15mm,Paolo 12mm,Paolo 15mm,Q Rubber 13-14mm"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Multilop 12mm,Multilop 15mm,Paolo 12mm,Paolo 15mm,Q Rubber 13-14mm"</formula1>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Simple,Media,Compleja"</formula1>
     </dataValidation>
-    <dataValidation sqref="B39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Paolo 9mm,Q Rubber 13mm"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1498,10 +1638,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="105" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1512,79 +1652,100 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>FUENTE: 3 fotos de notas de costeo manuscritas compartidas por el usuario el 2026-07-21 (Felpudos Mixtos / Piso Antifatiga, Felpudo Vinilo con Logo, Felpudo Vinilo en Rollos). Las fotos no quedaron guardadas como archivo en este repo (se compartieron pegadas en el chat, no como adjunto) — si se quiere conservar el original, hay que reenviarlas como archivo adjunto.</t>
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>FUENTE: 3 fotos de notas de costeo manuscritas compartidas por el usuario el 2026-07-21 (Felpudos Mixtos / Piso Antifatiga, Felpudo Vinilo con Logo, Felpudo Vinilo en Rollos). Las fotos no quedaron guardadas como archivo en este repo (se compartieron pegadas en el chat, no como adjunto).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>CÓMO SE DERIVARON LAS FÓRMULAS</t>
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>CAMBIOS EN ESTA VERSIÓN (v2)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Los valores en 'Datos Base' se obtuvieron por ingeniería inversa de los 4 (con logo) y 3 (mixtos) ejemplos manuscritos, ajustando una relación lineal (Costo = fijo + variable × área). El ajuste coincide casi exacto con los ejemplos de 'con logo' (diferencias de centavos por redondeo manual). En 'mixtos' el ajuste es un poco menos preciso (solo 3 puntos de datos) — validar con más ejemplos reales antes de confiar en el resultado para cotizaciones grandes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>SUPUESTOS A VALIDAR CON EL USUARIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>1. Longitud extra (ribete) en 'con logo': se asumió 0.20 m para áreas menores a 1.00 m² y 0.30 m para el resto, porque así calzan los 4 ejemplos dados. No está confirmado si la regla real depende del área, del ancho del logo, o de otra cosa — pedir más ejemplos con distintos tamaños de logo.</t>
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>1. La marca y espesor de la base ahora se elige SIEMPRE (con o sin logo), no solo cuando no lleva logo. Se unificó una sola tabla de materiales en S//m², convirtiendo los precios de rollo (S//m lineal) a S//m² dividiendo entre el ancho fijo del rollo (1.20 m) — supuesto a validar: asume que cortar un ancho menor al del rollo completo cuesta proporcionalmente lo mismo por m².</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>2. Se agregó 'Complejidad del logo' (Simple / Media / Compleja) como factor independiente del tamaño, con multiplicadores propios sobre costo de material extra y mano de obra. Solo el nivel 'Media' está calibrado con datos reales (los 4 ejemplos manuscritos). Simple y Compleja son ESTIMACIONES (marcadas en ámbar en 'Datos Base', sección 1b) — deben ajustarse en cuanto haya ejemplos reales de logos simples vs. complejos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>CÓMO SE DERIVARON LAS FÓRMULAS ORIGINALES (nivel 'Media')</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>2. Ajuste fijo de acabado ('tapiz'): en las notas originales varía entre S/23 y S/25 según el ejemplo. Se usó S/25 como estándar en el cotizador — confirmar si esa variación fue error de redondeo o un criterio real (p.ej. tamaño de logo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>3. Paolo 15mm: en la sección de COSTOS de la foto 3 aparece como S/90.00, pero en la sección de VENTA el cálculo del precio (S/158.00) solo cuadra si el costo es S/95.00. Se usó S/95.00 (el que sí reproduce el precio de venta anotado) — confirmar cuál es el costo correcto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>4. Mano de obra de 'Felpudos Mixtos': interpolada linealmente con solo 3 puntos de datos (S/40, S/45, S/50 para 1.20, 1.60 y 1.80 m de ancho) — es la fórmula menos confiable del archivo.</t>
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Los valores base se obtuvieron por ingeniería inversa de los 4 (con logo) y 3 (mixtos) ejemplos manuscritos, ajustando una relación lineal (Costo = fijo + variable × área). El ajuste coincide casi exacto con los ejemplos de 'con logo' (diferencias de centavos por redondeo manual). En 'mixtos' el ajuste es un poco menos preciso (solo 3 puntos de datos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>OTROS SUPUESTOS A VALIDAR CON EL USUARIO</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>5. Piso Antifatiga: solo hay 1 ejemplo de precio por marca/espesor (a 1.50×0.90m), así que el costo por m² es una simple división — no hay forma de confirmar si escala igual a otros tamaños.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>3. Longitud extra (ribete) en 'con logo': se asumió 0.20 m para áreas menores a 1.00 m² y 0.30 m para el resto. No está confirmado si la regla real depende del área, del tamaño del logo, o de la complejidad — con más ejemplos se podría fusionar este concepto con el factor de complejidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>4. Ajuste fijo de acabado ('tapiz'): varía entre S/23 y S/25 en las notas originales. Se usó S/25 como estándar, sin ligarlo a la complejidad — confirmar si debería variar por complejidad también.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>5. Paolo 15mm: en la sección de COSTOS de la foto 3 aparece como S/90.00, pero el cálculo de VENTA (S/158.00) solo cuadra si el costo es S/95.00. Se usó S/95.00 — confirmar cuál es correcto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>6. Mano de obra de 'Felpudos Mixtos': interpolada linealmente con solo 3 puntos de datos — es la fórmula menos confiable del archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>7. Piso Antifatiga: solo hay 1 ejemplo de precio por marca/espesor (a 1.50×0.90m) — no hay forma de confirmar si el costo por m² escala igual a otros tamaños.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>CÓMO USAR EL COTIZADOR</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>En la pestaña 'Cotizador', llenar solo las celdas amarillas (ancho, alto, si lleva logo, marca/espesor cuando aplique, y margen deseado — dejar el margen en blanco para usar el sugerido). El precio se recalcula solo. Si se actualiza algún costo real (p.ej. sube el precio del rollo), actualizarlo en 'Datos Base' y todo el cotizador se ajusta automáticamente.</t>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>En la pestaña 'Cotizador', llenar solo las celdas amarillas. El precio se recalcula solo. Si se actualiza algún costo real o se calibran los multiplicadores de complejidad, actualizarlo en 'Datos Base' y todo el cotizador se ajusta automáticamente.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten logo complexity multipliers to 0.8x/1.2x per user feedback
</commit_message>
<xml_diff>
--- a/contexto-marcas/felpudos-y-servicios/herramientas/Felpudos_Cotizador.xlsx
+++ b/contexto-marcas/felpudos-y-servicios/herramientas/Felpudos_Cotizador.xlsx
@@ -816,14 +816,14 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>ESTIMADO — sin datos reales. Ajustar cuando haya ejemplos (1-2 colores, texto simple).</t>
+          <t>ESTIMADO (ajustado por el usuario) — sin datos reales aún. Ajustar cuando haya ejemplos (1-2 colores, texto simple).</t>
         </is>
       </c>
     </row>
@@ -852,14 +852,14 @@
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>ESTIMADO — sin datos reales. Ajustar cuando haya ejemplos (4+ colores, degradados, detalle fino).</t>
+          <t>ESTIMADO (ajustado por el usuario) — sin datos reales aún. Ajustar cuando haya ejemplos (4+ colores, degradados, detalle fino).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace labor cost formula with 4 fixed levels per user correction
Mano de obra for Felpudo con Logo no longer uses a size-derived linear
formula. The user pays 4 flat levels in practice based on their own
combined judgment of size + complexity (S/100, S/120, S/150, S/180),
selected manually in the Cotizador rather than computed. Complexity
multiplier now only affects the logo material-extra cost, not labor.
</commit_message>
<xml_diff>
--- a/contexto-marcas/felpudos-y-servicios/herramientas/Felpudos_Cotizador.xlsx
+++ b/contexto-marcas/felpudos-y-servicios/herramientas/Felpudos_Cotizador.xlsx
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -781,7 +781,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>1b. FELPUDO DE VINILO — NIVELES DE COMPLEJIDAD DEL LOGO (solo si lleva logo)</t>
+          <t>1b. FELPUDO DE VINILO — COMPLEJIDAD DEL LOGO (afecta costo de material extra; solo si lleva logo)</t>
         </is>
       </c>
     </row>
@@ -796,11 +796,7 @@
           <t>Mult. costo material extra</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Mult. mano de obra</t>
-        </is>
-      </c>
+      <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="4" t="inlineStr"/>
       <c r="E14" s="4" t="inlineStr"/>
       <c r="F14" s="4" t="inlineStr">
@@ -818,9 +814,6 @@
       <c r="B15" s="9" t="n">
         <v>0.8</v>
       </c>
-      <c r="C15" s="9" t="n">
-        <v>0.8</v>
-      </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
           <t>ESTIMADO (ajustado por el usuario) — sin datos reales aún. Ajustar cuando haya ejemplos (1-2 colores, texto simple).</t>
@@ -836,9 +829,6 @@
       <c r="B16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Baseline = los 4 ejemplos reales que sí tenemos (logos con 2-3 colores, tipo Vet.Orbegoso/FINA/Bar Popular).</t>
@@ -854,9 +844,6 @@
       <c r="B17" s="9" t="n">
         <v>1.2</v>
       </c>
-      <c r="C17" s="9" t="n">
-        <v>1.2</v>
-      </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
           <t>ESTIMADO (ajustado por el usuario) — sin datos reales aún. Ajustar cuando haya ejemplos (4+ colores, degradados, detalle fino).</t>
@@ -866,316 +853,382 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>1c. FELPUDO DE VINILO — OTROS COSTOS DEL LOGO (nivel 'Media', antes de multiplicador)</t>
+          <t>1c. FELPUDO DE VINILO — NIVELES DE MANO DE OBRA (pago por felpudo, según tamaño y complejidad juntos; solo si lleva logo)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Concepto</t>
+          <t>Nivel</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Unidad</t>
+          <t>Pago (S/)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Nota</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Costo material extra ribete (por m lineal)</t>
+          <t>Nivel 1</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>94.90000000000001</v>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>S//m</t>
+        <v>100</v>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Tamaño chico / complejidad baja</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Longitud extra si área &lt; 1.00 m²</t>
+          <t>Nivel 2</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>m</t>
+        <v>120</v>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Tamaño mediano o complejidad media</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Longitud extra si área ≥ 1.00 m²</t>
+          <t>Nivel 3</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>m</t>
+        <v>150</v>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Tamaño grande o complejidad alta</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Mano de obra — componente fijo</t>
+          <t>Nivel 4</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>80</v>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>S/</t>
+        <v>180</v>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Tamaño grande + complejidad alta juntos</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Mano de obra — componente variable</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="n">
-        <v>37.04</v>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>S//m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Ajuste fijo de acabado (tapiz)</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>S/</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>2. FELPUDOS MIXTOS (retienen polvo y secan, perfil de jebe — marca base Confort Mat)</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>El usuario asigna el Nivel manualmente según su propio criterio de tamaño + complejidad combinados — no hay una regla automática que lo derive de ancho/alto. Elegir el nivel en el Cotizador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>1d. FELPUDO DE VINILO — OTROS COSTOS DEL LOGO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Unidad</t>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Costo material extra ribete (por m lineal)</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>S//m</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Costo material</t>
+          <t>Longitud extra si área &lt; 1.00 m²</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>45</v>
+        <v>0.2</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>S//m²</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Costo perfil (ribete de jebe)</t>
+          <t>Longitud extra si área ≥ 1.00 m²</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>9</v>
+        <v>0.3</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>S//m</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>Ajuste fijo de acabado (tapiz)</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>S/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2. FELPUDOS MIXTOS (retienen polvo y secan, perfil de jebe — marca base Confort Mat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Costo material</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>S//m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Costo perfil (ribete de jebe)</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>S//m</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
           <t>Extra fijo sobre perímetro</t>
         </is>
       </c>
-      <c r="B32" s="6" t="n">
+      <c r="B38" s="6" t="n">
         <v>0.24</v>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Mano de obra — componente fijo</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>S/</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Mano de obra — componente variable</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="n">
-        <v>16.67</v>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>S//m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Margen sugerido</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="n">
-        <v>0.33</v>
-      </c>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>3. PISO ANTIFATIGA</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Espesor</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Costo (S//m²)</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Margen sugerido</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr"/>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>Clave</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Paolo</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>9mm</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="n">
-        <v>37.04</v>
-      </c>
-      <c r="D39" s="7" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>Paolo 9mm</t>
+          <t>Mano de obra — componente fijo</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>S/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
+          <t>Mano de obra — componente variable</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>S//m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Margen sugerido</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>3. PISO ANTIFATIGA</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Espesor</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Costo (S//m²)</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Margen sugerido</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Clave</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Paolo</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>9mm</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>37.04</v>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Paolo 9mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
           <t>Q Rubber</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>13mm</t>
         </is>
       </c>
-      <c r="C40" s="6" t="n">
+      <c r="C46" s="6" t="n">
         <v>87.41</v>
       </c>
-      <c r="D40" s="7" t="n">
+      <c r="D46" s="7" t="n">
         <v>0.41</v>
       </c>
-      <c r="F40" s="5" t="inlineStr">
+      <c r="F46" s="5" t="inlineStr">
         <is>
           <t>Q Rubber 13mm</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A34:F34"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1187,7 +1240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1208,7 +1261,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Llena solo las celdas amarillas. Las celdas ámbar en 'Datos Base' (niveles de complejidad Simple/Compleja) son estimaciones — ajústalas ahí cuando tengas datos reales.</t>
+          <t>Llena solo las celdas amarillas. El Nivel de mano de obra (1-4) lo eliges tú a mano según tamaño + complejidad combinados. Las celdas ámbar en 'Datos Base' (complejidad Simple/Compleja del material) son estimaciones — ajústalas ahí cuando tengas datos reales.</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1319,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Complejidad del logo (solo si lleva logo)</t>
+          <t>Complejidad del logo (material — solo si lleva logo)</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
@@ -1278,343 +1331,355 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>Nivel de mano de obra 1-4 (solo si lleva logo)</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
           <t>Margen deseado (%) — vacío = usar el sugerido</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="B11" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>RESULTADOS</t>
         </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Área (m²)</t>
-        </is>
-      </c>
-      <c r="B13" s="14">
-        <f>B5*B6</f>
-        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Costo material base (S/)</t>
-        </is>
-      </c>
-      <c r="B14" s="15">
-        <f>B13*INDEX('Datos Base'!$C$6:$C$11,MATCH(B7,'Datos Base'!$F$6:$F$11,0))</f>
+          <t>Área (m²)</t>
+        </is>
+      </c>
+      <c r="B14" s="14">
+        <f>B5*B6</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Costo material extra por logo (S/)</t>
+          <t>Costo material base (S/)</t>
         </is>
       </c>
       <c r="B15" s="15">
-        <f>IF(B8="Sí", IF(B13&lt;1,'Datos Base'!$B$22,'Datos Base'!$B$23)*'Datos Base'!$B$21*INDEX('Datos Base'!$B$15:$B$17,MATCH(B9,'Datos Base'!$A$15:$A$17,0)), 0)</f>
+        <f>B14*INDEX('Datos Base'!$C$6:$C$11,MATCH(B7,'Datos Base'!$F$6:$F$11,0))</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Costo mano de obra (S/)</t>
+          <t>Costo material extra por logo (S/)</t>
         </is>
       </c>
       <c r="B16" s="15">
-        <f>IF(B8="Sí", ('Datos Base'!$B$24+'Datos Base'!$B$25*B13)*INDEX('Datos Base'!$C$15:$C$17,MATCH(B9,'Datos Base'!$A$15:$A$17,0)), 0)</f>
+        <f>IF(B8="Sí", IF(B14&lt;1,'Datos Base'!$B$30,'Datos Base'!$B$31)*'Datos Base'!$B$29*INDEX('Datos Base'!$B$15:$B$17,MATCH(B9,'Datos Base'!$A$15:$A$17,0)), 0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Costo total (S/)</t>
+          <t>Costo mano de obra (S/)</t>
         </is>
       </c>
       <c r="B17" s="15">
-        <f>B14+B15+B16</f>
+        <f>IF(B8="Sí", INDEX('Datos Base'!$B$21:$B$24,MATCH(B10,'Datos Base'!$A$21:$A$24,0)), 0)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Margen aplicado (%)</t>
-        </is>
-      </c>
-      <c r="B18" s="16">
-        <f>IF(B10&lt;&gt;"", B10, INDEX('Datos Base'!$D$6:$D$11,MATCH(B7,'Datos Base'!$F$6:$F$11,0)))</f>
+          <t>Costo total (S/)</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>B15+B16+B17</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
+          <t>Margen aplicado (%)</t>
+        </is>
+      </c>
+      <c r="B19" s="16">
+        <f>IF(B11&lt;&gt;"", B11, INDEX('Datos Base'!$D$6:$D$11,MATCH(B7,'Datos Base'!$F$6:$F$11,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
           <t>Ajuste fijo de acabado (S/, solo con logo)</t>
         </is>
       </c>
-      <c r="B19" s="15">
-        <f>IF(B8="Sí",'Datos Base'!$B$26,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="B20" s="15">
+        <f>IF(B8="Sí",'Datos Base'!$B$32,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>PRECIO SUGERIDO (S/)</t>
         </is>
       </c>
-      <c r="B20" s="17">
-        <f>ROUND(B17/(1-B18)+B19,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="B21" s="17">
+        <f>ROUND(B18/(1-B19)+B20,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>B. FELPUDOS MIXTOS</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Ancho (m)</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="n">
-        <v>1.2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Alto / largo (m)</t>
+          <t>Ancho (m)</t>
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
+          <t>Alto / largo (m)</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
           <t>Margen deseado (%) — vacío = usar el sugerido</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="B27" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>RESULTADOS</t>
         </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Área (m²)</t>
-        </is>
-      </c>
-      <c r="B29" s="14">
-        <f>B24*B25</f>
-        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Perímetro + extra (m)</t>
+          <t>Área (m²)</t>
         </is>
       </c>
       <c r="B30" s="14">
-        <f>2*(B24+B25)+'Datos Base'!$B$32</f>
+        <f>B25*B26</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Costo materiales (S/)</t>
-        </is>
-      </c>
-      <c r="B31" s="15">
-        <f>B29*'Datos Base'!$B$30+B30*'Datos Base'!$B$31</f>
+          <t>Perímetro + extra (m)</t>
+        </is>
+      </c>
+      <c r="B31" s="14">
+        <f>2*(B25+B26)+'Datos Base'!$B$38</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Costo mano de obra (S/)</t>
+          <t>Costo materiales (S/)</t>
         </is>
       </c>
       <c r="B32" s="15">
-        <f>'Datos Base'!$B$33+'Datos Base'!$B$34*B29</f>
+        <f>B30*'Datos Base'!$B$36+B31*'Datos Base'!$B$37</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Costo total (S/)</t>
+          <t>Costo mano de obra (S/)</t>
         </is>
       </c>
       <c r="B33" s="15">
-        <f>B31+B32</f>
+        <f>'Datos Base'!$B$39+'Datos Base'!$B$40*B30</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
+          <t>Costo total (S/)</t>
+        </is>
+      </c>
+      <c r="B34" s="15">
+        <f>B32+B33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
           <t>Margen aplicado (%)</t>
         </is>
       </c>
-      <c r="B34" s="16">
-        <f>IF(B26&lt;&gt;"",B26,'Datos Base'!$B$35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="B35" s="16">
+        <f>IF(B27&lt;&gt;"",B27,'Datos Base'!$B$41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>PRECIO SUGERIDO (S/)</t>
         </is>
       </c>
-      <c r="B35" s="17">
-        <f>ROUND(B33/(1-B34),2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="B36" s="17">
+        <f>ROUND(B34/(1-B35),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>C. PISO ANTIFATIGA</t>
         </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>Ancho (m)</t>
-        </is>
-      </c>
-      <c r="B39" s="12" t="n">
-        <v>1.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Alto / largo (m)</t>
+          <t>Ancho (m)</t>
         </is>
       </c>
       <c r="B40" s="12" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Marca y espesor</t>
-        </is>
-      </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>Paolo 9mm</t>
-        </is>
+          <t>Alto / largo (m)</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="n">
+        <v>0.9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
+          <t>Marca y espesor</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Paolo 9mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
           <t>Margen deseado (%) — vacío = usar el sugerido</t>
         </is>
       </c>
-      <c r="B42" s="7" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+      <c r="B43" s="7" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>RESULTADOS</t>
         </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Área (m²)</t>
-        </is>
-      </c>
-      <c r="B45" s="14">
-        <f>B39*B40</f>
-        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Costo por m² (S/)</t>
-        </is>
-      </c>
-      <c r="B46" s="15">
-        <f>INDEX('Datos Base'!$C$39:$C$40,MATCH(B41,'Datos Base'!$F$39:$F$40,0))</f>
+          <t>Área (m²)</t>
+        </is>
+      </c>
+      <c r="B46" s="14">
+        <f>B40*B41</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Costo total (S/)</t>
+          <t>Costo por m² (S/)</t>
         </is>
       </c>
       <c r="B47" s="15">
-        <f>B45*B46</f>
+        <f>INDEX('Datos Base'!$C$45:$C$46,MATCH(B42,'Datos Base'!$F$45:$F$46,0))</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
+          <t>Costo total (S/)</t>
+        </is>
+      </c>
+      <c r="B48" s="15">
+        <f>B46*B47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
           <t>Margen aplicado (%)</t>
         </is>
       </c>
-      <c r="B48" s="16">
-        <f>IF(B42&lt;&gt;"",B42,INDEX('Datos Base'!$D$39:$D$40,MATCH(B41,'Datos Base'!$F$39:$F$40,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="B49" s="16">
+        <f>IF(B43&lt;&gt;"",B43,INDEX('Datos Base'!$D$45:$D$46,MATCH(B42,'Datos Base'!$F$45:$F$46,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>PRECIO SUGERIDO (S/)</t>
         </is>
       </c>
-      <c r="B49" s="17">
-        <f>ROUND(B47/(1-B48),2)</f>
+      <c r="B50" s="17">
+        <f>ROUND(B48/(1-B49),2)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A39:F39"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Confort Mat 14-15mm,Multilop 12mm,Multilop 15mm,Paolo 12mm,Paolo 15mm,Q Rubber 13-14mm"</formula1>
     </dataValidation>
@@ -1624,7 +1689,10 @@
     <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Simple,Media,Compleja"</formula1>
     </dataValidation>
-    <dataValidation sqref="B41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Nivel 1,Nivel 2,Nivel 3,Nivel 4"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Paolo 9mm,Q Rubber 13mm"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1638,7 +1706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
@@ -1661,7 +1729,7 @@
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>CAMBIOS EN ESTA VERSIÓN (v2)</t>
+          <t>CAMBIOS EN ESTA VERSIÓN (v3)</t>
         </is>
       </c>
     </row>
@@ -1675,75 +1743,82 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>2. Se agregó 'Complejidad del logo' (Simple / Media / Compleja) como factor independiente del tamaño, con multiplicadores propios sobre costo de material extra y mano de obra. Solo el nivel 'Media' está calibrado con datos reales (los 4 ejemplos manuscritos). Simple y Compleja son ESTIMACIONES (marcadas en ámbar en 'Datos Base', sección 1b) — deben ajustarse en cuanto haya ejemplos reales de logos simples vs. complejos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
+          <t>2. Se agregó 'Complejidad del logo' (Simple ×0.8 / Media ×1.0 / Compleja ×1.2) como factor independiente del tamaño, que afecta SOLO el costo de material extra. Solo el nivel 'Media' está calibrado con datos reales (los 4 ejemplos manuscritos); Simple y Compleja son ESTIMACIONES (marcadas en ámbar en 'Datos Base', sección 1b) — deben ajustarse en cuanto haya ejemplos reales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>3. La mano de obra de 'Felpudo con Logo' YA NO se calcula con una fórmula (fijo + variable×área) — el usuario indicó que en la práctica paga 4 niveles fijos según tamaño y complejidad combinados: Nivel 1 = S/100, Nivel 2 = S/120, Nivel 3 = S/150, Nivel 4 = S/180 (Datos Base, sección 1c). El nivel se elige a mano en el Cotizador — no hay una regla automática que lo derive de ancho/alto, porque el usuario junta tamaño y complejidad en un solo criterio de su propio juicio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>CÓMO SE DERIVARON LAS FÓRMULAS ORIGINALES (nivel 'Media')</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Los valores base se obtuvieron por ingeniería inversa de los 4 (con logo) y 3 (mixtos) ejemplos manuscritos, ajustando una relación lineal (Costo = fijo + variable × área). El ajuste coincide casi exacto con los ejemplos de 'con logo' (diferencias de centavos por redondeo manual). En 'mixtos' el ajuste es un poco menos preciso (solo 3 puntos de datos).</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>OTROS SUPUESTOS A VALIDAR CON EL USUARIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>3. Longitud extra (ribete) en 'con logo': se asumió 0.20 m para áreas menores a 1.00 m² y 0.30 m para el resto. No está confirmado si la regla real depende del área, del tamaño del logo, o de la complejidad — con más ejemplos se podría fusionar este concepto con el factor de complejidad.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>4. Ajuste fijo de acabado ('tapiz'): varía entre S/23 y S/25 en las notas originales. Se usó S/25 como estándar, sin ligarlo a la complejidad — confirmar si debería variar por complejidad también.</t>
+          <t>3. Longitud extra (ribete) en 'con logo': se asumió 0.20 m para áreas menores a 1.00 m² y 0.30 m para el resto. No está confirmado si la regla real depende del área, del tamaño del logo, o de la complejidad — con más ejemplos se podría fusionar este concepto con el factor de complejidad.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>5. Paolo 15mm: en la sección de COSTOS de la foto 3 aparece como S/90.00, pero el cálculo de VENTA (S/158.00) solo cuadra si el costo es S/95.00. Se usó S/95.00 — confirmar cuál es correcto.</t>
+          <t>4. Ajuste fijo de acabado ('tapiz'): varía entre S/23 y S/25 en las notas originales. Se usó S/25 como estándar, sin ligarlo a la complejidad — confirmar si debería variar por complejidad también.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t>6. Mano de obra de 'Felpudos Mixtos': interpolada linealmente con solo 3 puntos de datos — es la fórmula menos confiable del archivo.</t>
+          <t>5. Paolo 15mm: en la sección de COSTOS de la foto 3 aparece como S/90.00, pero el cálculo de VENTA (S/158.00) solo cuadra si el costo es S/95.00. Se usó S/95.00 — confirmar cuál es correcto.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
+          <t>6. Mano de obra de 'Felpudos Mixtos': interpolada linealmente con solo 3 puntos de datos — es la fórmula menos confiable del archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
           <t>7. Piso Antifatiga: solo hay 1 ejemplo de precio por marca/espesor (a 1.50×0.90m) — no hay forma de confirmar si el costo por m² escala igual a otros tamaños.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="19" t="inlineStr">
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>CÓMO USAR EL COTIZADOR</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>En la pestaña 'Cotizador', llenar solo las celdas amarillas. El precio se recalcula solo. Si se actualiza algún costo real o se calibran los multiplicadores de complejidad, actualizarlo en 'Datos Base' y todo el cotizador se ajusta automáticamente.</t>
         </is>

</xml_diff>

<commit_message>
Simplify logo pricing: material by size only, labor by complexity only
Per user correction: complexity should never have affected material
cost (that's tied to size alone) — it should only drive labor. Removes
the earlier 4-level combined size+complexity labor table and the
material complexity multiplier. Now: material extra = f(tamaño) via
ribete length x Multilop 12mm rate; mano de obra = f(complejidad) via
3 flat rates (Simple S/100, Media S/120, Compleja S/150).
</commit_message>
<xml_diff>
--- a/contexto-marcas/felpudos-y-servicios/herramientas/Felpudos_Cotizador.xlsx
+++ b/contexto-marcas/felpudos-y-servicios/herramientas/Felpudos_Cotizador.xlsx
@@ -18,12 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="166" formatCode="&quot;S/&quot; #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;S/&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,15 +61,8 @@
       <name val="Arial"/>
       <color rgb="000000FF"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <i val="1"/>
-      <color rgb="00CC0000"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -90,11 +82,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
     <fill>
@@ -129,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -151,15 +138,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -169,13 +147,13 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -549,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -781,7 +759,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>1b. FELPUDO DE VINILO — COMPLEJIDAD DEL LOGO (afecta costo de material extra; solo si lleva logo)</t>
+          <t>1b. FELPUDO DE VINILO — COMPLEJIDAD DEL LOGO (afecta la mano de obra; solo si lleva logo)</t>
         </is>
       </c>
     </row>
@@ -793,7 +771,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Mult. costo material extra</t>
+          <t>Pago mano de obra (S/)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
@@ -811,12 +789,12 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>ESTIMADO (ajustado por el usuario) — sin datos reales aún. Ajustar cuando haya ejemplos (1-2 colores, texto simple).</t>
+      <c r="B15" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Logo de 1-2 colores, diseño básico.</t>
         </is>
       </c>
     </row>
@@ -826,12 +804,12 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
-        <v>1</v>
+      <c r="B16" s="6" t="n">
+        <v>120</v>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Baseline = los 4 ejemplos reales que sí tenemos (logos con 2-3 colores, tipo Vet.Orbegoso/FINA/Bar Popular).</t>
+          <t>Baseline — coincide con el ejemplo real 1.20×0.90m (Vet. Orbegoso).</t>
         </is>
       </c>
     </row>
@@ -841,113 +819,110 @@
           <t>Compleja</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>ESTIMADO (ajustado por el usuario) — sin datos reales aún. Ajustar cuando haya ejemplos (4+ colores, degradados, detalle fino).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>1c. FELPUDO DE VINILO — NIVELES DE MANO DE OBRA (pago por felpudo, según tamaño y complejidad juntos; solo si lleva logo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Nivel</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Pago (S/)</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr"/>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="inlineStr"/>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Nota</t>
+      <c r="B17" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Logo con muchos colores / detalle fino (ej. diseño tipo FINA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>El material extra del logo (sección 1c) NO depende de la complejidad — solo del tamaño del felpudo. La complejidad mueve únicamente el costo de mano de obra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>1c. FELPUDO DE VINILO — MATERIAL EXTRA DEL LOGO (depende solo del tamaño)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Nivel 1</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Tamaño chico / complejidad baja</t>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Nivel 2</t>
+          <t>Costo material extra ribete (por m lineal)</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>120</v>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Tamaño mediano o complejidad media</t>
+        <v>94.90000000000001</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>S//m</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Nivel 3</t>
+          <t>Longitud extra si área &lt; 1.00 m²</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>150</v>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Tamaño grande o complejidad alta</t>
+        <v>0.2</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Nivel 4</t>
+          <t>Longitud extra si área ≥ 1.00 m²</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>Tamaño grande + complejidad alta juntos</t>
+        <v>0.3</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>El usuario asigna el Nivel manualmente según su propio criterio de tamaño + complejidad combinados — no hay una regla automática que lo derive de ancho/alto. Elegir el nivel en el Cotizador.</t>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Ajuste fijo de acabado (tapiz)</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>S/</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>1d. FELPUDO DE VINILO — OTROS COSTOS DEL LOGO</t>
+          <t>2. FELPUDOS MIXTOS (retienen polvo y secan, perfil de jebe — marca base Confort Mat)</t>
         </is>
       </c>
     </row>
@@ -971,41 +946,41 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Costo material extra ribete (por m lineal)</t>
+          <t>Costo material</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>94.90000000000001</v>
+        <v>45</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>S//m</t>
+          <t>S//m²</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Longitud extra si área &lt; 1.00 m²</t>
+          <t>Costo perfil (ribete de jebe)</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0.2</v>
+        <v>9</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>S//m</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Longitud extra si área ≥ 1.00 m²</t>
+          <t>Extra fijo sobre perímetro</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.3</v>
+        <v>0.24</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
@@ -1016,11 +991,11 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Ajuste fijo de acabado (tapiz)</t>
+          <t>Mano de obra — componente fijo</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
@@ -1028,207 +1003,122 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>2. FELPUDOS MIXTOS (retienen polvo y secan, perfil de jebe — marca base Confort Mat)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Costo material</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Mano de obra — componente variable</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>S//m²</t>
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Margen sugerido</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>3. PISO ANTIFATIGA</t>
+        </is>
+      </c>
+    </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Costo perfil (ribete de jebe)</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>S//m</t>
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Espesor</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Costo (S//m²)</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Margen sugerido</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Clave</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Extra fijo sobre perímetro</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>m</t>
+          <t>Paolo</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>9mm</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>37.04</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Paolo 9mm</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Mano de obra — componente fijo</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>S/</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>Mano de obra — componente variable</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="n">
-        <v>16.67</v>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>S//m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Margen sugerido</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="n">
-        <v>0.33</v>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>3. PISO ANTIFATIGA</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Espesor</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Costo (S//m²)</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Margen sugerido</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr"/>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>Clave</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Paolo</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>9mm</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="n">
-        <v>37.04</v>
-      </c>
-      <c r="D45" s="7" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>Paolo 9mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
           <t>Q Rubber</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>13mm</t>
         </is>
       </c>
-      <c r="C46" s="6" t="n">
+      <c r="C39" s="6" t="n">
         <v>87.41</v>
       </c>
-      <c r="D46" s="7" t="n">
+      <c r="D39" s="7" t="n">
         <v>0.41</v>
       </c>
-      <c r="F46" s="5" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>Q Rubber 13mm</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A36:F36"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A18:F18"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A43:F43"/>
+    <mergeCell ref="A20:F20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1240,7 +1130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1261,7 +1151,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Llena solo las celdas amarillas. El Nivel de mano de obra (1-4) lo eliges tú a mano según tamaño + complejidad combinados. Las celdas ámbar en 'Datos Base' (complejidad Simple/Compleja del material) son estimaciones — ajústalas ahí cuando tengas datos reales.</t>
+          <t>Llena solo las celdas amarillas. La Complejidad del logo determina la mano de obra (Simple=S/100 / Media=S/120 / Compleja=S/150); el material extra del logo depende solo del tamaño.</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1168,7 @@
           <t>Ancho (m)</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="9" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -1288,7 +1178,7 @@
           <t>Alto / largo (m)</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.9</v>
       </c>
     </row>
@@ -1298,7 +1188,7 @@
           <t>Marca y espesor de la base</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Confort Mat 14-15mm</t>
         </is>
@@ -1310,7 +1200,7 @@
           <t>¿Lleva logo?</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1319,10 +1209,10 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Complejidad del logo (material — solo si lleva logo)</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
+          <t>Complejidad del logo (define la mano de obra — solo si lleva logo)</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
@@ -1331,355 +1221,343 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Nivel de mano de obra 1-4 (solo si lleva logo)</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Nivel 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
           <t>Margen deseado (%) — vacío = usar el sugerido</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>RESULTADOS</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>RESULTADOS</t>
-        </is>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Área (m²)</t>
+        </is>
+      </c>
+      <c r="B13" s="11">
+        <f>B5*B6</f>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Área (m²)</t>
-        </is>
-      </c>
-      <c r="B14" s="14">
-        <f>B5*B6</f>
+          <t>Costo material base (S/)</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>B13*INDEX('Datos Base'!$C$6:$C$11,MATCH(B7,'Datos Base'!$F$6:$F$11,0))</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Costo material base (S/)</t>
-        </is>
-      </c>
-      <c r="B15" s="15">
-        <f>B14*INDEX('Datos Base'!$C$6:$C$11,MATCH(B7,'Datos Base'!$F$6:$F$11,0))</f>
+          <t>Costo material extra por logo (S/, solo según tamaño)</t>
+        </is>
+      </c>
+      <c r="B15" s="12">
+        <f>IF(B8="Sí", IF(B13&lt;1,'Datos Base'!$B$23,'Datos Base'!$B$24)*'Datos Base'!$B$22, 0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Costo material extra por logo (S/)</t>
-        </is>
-      </c>
-      <c r="B16" s="15">
-        <f>IF(B8="Sí", IF(B14&lt;1,'Datos Base'!$B$30,'Datos Base'!$B$31)*'Datos Base'!$B$29*INDEX('Datos Base'!$B$15:$B$17,MATCH(B9,'Datos Base'!$A$15:$A$17,0)), 0)</f>
+          <t>Costo mano de obra (S/, según complejidad)</t>
+        </is>
+      </c>
+      <c r="B16" s="12">
+        <f>IF(B8="Sí", INDEX('Datos Base'!$B$15:$B$17,MATCH(B9,'Datos Base'!$A$15:$A$17,0)), 0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Costo mano de obra (S/)</t>
-        </is>
-      </c>
-      <c r="B17" s="15">
-        <f>IF(B8="Sí", INDEX('Datos Base'!$B$21:$B$24,MATCH(B10,'Datos Base'!$A$21:$A$24,0)), 0)</f>
+          <t>Costo total (S/)</t>
+        </is>
+      </c>
+      <c r="B17" s="12">
+        <f>B14+B15+B16</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Costo total (S/)</t>
-        </is>
-      </c>
-      <c r="B18" s="15">
-        <f>B15+B16+B17</f>
+          <t>Margen aplicado (%)</t>
+        </is>
+      </c>
+      <c r="B18" s="13">
+        <f>IF(B10&lt;&gt;"", B10, INDEX('Datos Base'!$D$6:$D$11,MATCH(B7,'Datos Base'!$F$6:$F$11,0)))</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Margen aplicado (%)</t>
-        </is>
-      </c>
-      <c r="B19" s="16">
-        <f>IF(B11&lt;&gt;"", B11, INDEX('Datos Base'!$D$6:$D$11,MATCH(B7,'Datos Base'!$F$6:$F$11,0)))</f>
+          <t>Ajuste fijo de acabado (S/, solo con logo)</t>
+        </is>
+      </c>
+      <c r="B19" s="12">
+        <f>IF(B8="Sí",'Datos Base'!$B$25,0)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Ajuste fijo de acabado (S/, solo con logo)</t>
-        </is>
-      </c>
-      <c r="B20" s="15">
-        <f>IF(B8="Sí",'Datos Base'!$B$32,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>PRECIO SUGERIDO (S/)</t>
         </is>
       </c>
-      <c r="B21" s="17">
-        <f>ROUND(B18/(1-B19)+B20,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="B20" s="14">
+        <f>ROUND(B17/(1-B18)+B19,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>B. FELPUDOS MIXTOS</t>
         </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Ancho (m)</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Ancho (m)</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="n">
-        <v>1.2</v>
+          <t>Alto / largo (m)</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Alto / largo (m)</t>
-        </is>
-      </c>
-      <c r="B26" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
           <t>Margen deseado (%) — vacío = usar el sugerido</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n"/>
+      <c r="B26" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>RESULTADOS</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>RESULTADOS</t>
-        </is>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Área (m²)</t>
+        </is>
+      </c>
+      <c r="B29" s="11">
+        <f>B24*B25</f>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Área (m²)</t>
-        </is>
-      </c>
-      <c r="B30" s="14">
-        <f>B25*B26</f>
+          <t>Perímetro + extra (m)</t>
+        </is>
+      </c>
+      <c r="B30" s="11">
+        <f>2*(B24+B25)+'Datos Base'!$B$31</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Perímetro + extra (m)</t>
-        </is>
-      </c>
-      <c r="B31" s="14">
-        <f>2*(B25+B26)+'Datos Base'!$B$38</f>
+          <t>Costo materiales (S/)</t>
+        </is>
+      </c>
+      <c r="B31" s="12">
+        <f>B29*'Datos Base'!$B$29+B30*'Datos Base'!$B$30</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Costo materiales (S/)</t>
-        </is>
-      </c>
-      <c r="B32" s="15">
-        <f>B30*'Datos Base'!$B$36+B31*'Datos Base'!$B$37</f>
+          <t>Costo mano de obra (S/)</t>
+        </is>
+      </c>
+      <c r="B32" s="12">
+        <f>'Datos Base'!$B$32+'Datos Base'!$B$33*B29</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Costo mano de obra (S/)</t>
-        </is>
-      </c>
-      <c r="B33" s="15">
-        <f>'Datos Base'!$B$39+'Datos Base'!$B$40*B30</f>
+          <t>Costo total (S/)</t>
+        </is>
+      </c>
+      <c r="B33" s="12">
+        <f>B31+B32</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Costo total (S/)</t>
-        </is>
-      </c>
-      <c r="B34" s="15">
-        <f>B32+B33</f>
+          <t>Margen aplicado (%)</t>
+        </is>
+      </c>
+      <c r="B34" s="13">
+        <f>IF(B26&lt;&gt;"",B26,'Datos Base'!$B$34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Margen aplicado (%)</t>
-        </is>
-      </c>
-      <c r="B35" s="16">
-        <f>IF(B27&lt;&gt;"",B27,'Datos Base'!$B$41)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>PRECIO SUGERIDO (S/)</t>
         </is>
       </c>
-      <c r="B36" s="17">
-        <f>ROUND(B34/(1-B35),2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="B35" s="14">
+        <f>ROUND(B33/(1-B34),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>C. PISO ANTIFATIGA</t>
         </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Ancho (m)</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Ancho (m)</t>
-        </is>
-      </c>
-      <c r="B40" s="12" t="n">
-        <v>1.5</v>
+          <t>Alto / largo (m)</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="n">
+        <v>0.9</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Alto / largo (m)</t>
-        </is>
-      </c>
-      <c r="B41" s="12" t="n">
-        <v>0.9</v>
+          <t>Marca y espesor</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Paolo 9mm</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Marca y espesor</t>
-        </is>
-      </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>Paolo 9mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
           <t>Margen deseado (%) — vacío = usar el sugerido</t>
         </is>
       </c>
-      <c r="B43" s="7" t="n"/>
+      <c r="B42" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>RESULTADOS</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>RESULTADOS</t>
-        </is>
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Área (m²)</t>
+        </is>
+      </c>
+      <c r="B45" s="11">
+        <f>B39*B40</f>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Área (m²)</t>
-        </is>
-      </c>
-      <c r="B46" s="14">
-        <f>B40*B41</f>
+          <t>Costo por m² (S/)</t>
+        </is>
+      </c>
+      <c r="B46" s="12">
+        <f>INDEX('Datos Base'!$C$38:$C$39,MATCH(B41,'Datos Base'!$F$38:$F$39,0))</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Costo por m² (S/)</t>
-        </is>
-      </c>
-      <c r="B47" s="15">
-        <f>INDEX('Datos Base'!$C$45:$C$46,MATCH(B42,'Datos Base'!$F$45:$F$46,0))</f>
+          <t>Costo total (S/)</t>
+        </is>
+      </c>
+      <c r="B47" s="12">
+        <f>B45*B46</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Costo total (S/)</t>
-        </is>
-      </c>
-      <c r="B48" s="15">
-        <f>B46*B47</f>
+          <t>Margen aplicado (%)</t>
+        </is>
+      </c>
+      <c r="B48" s="13">
+        <f>IF(B42&lt;&gt;"",B42,INDEX('Datos Base'!$D$38:$D$39,MATCH(B41,'Datos Base'!$F$38:$F$39,0)))</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Margen aplicado (%)</t>
-        </is>
-      </c>
-      <c r="B49" s="16">
-        <f>IF(B43&lt;&gt;"",B43,INDEX('Datos Base'!$D$45:$D$46,MATCH(B42,'Datos Base'!$F$45:$F$46,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>PRECIO SUGERIDO (S/)</t>
         </is>
       </c>
-      <c r="B50" s="17">
-        <f>ROUND(B48/(1-B49),2)</f>
+      <c r="B49" s="14">
+        <f>ROUND(B47/(1-B48),2)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A39:F39"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="4">
     <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Confort Mat 14-15mm,Multilop 12mm,Multilop 15mm,Paolo 12mm,Paolo 15mm,Q Rubber 13-14mm"</formula1>
     </dataValidation>
@@ -1689,10 +1567,7 @@
     <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Simple,Media,Compleja"</formula1>
     </dataValidation>
-    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Nivel 1,Nivel 2,Nivel 3,Nivel 4"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Paolo 9mm,Q Rubber 13mm"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1706,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
@@ -1720,105 +1595,98 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>FUENTE: 3 fotos de notas de costeo manuscritas compartidas por el usuario el 2026-07-21 (Felpudos Mixtos / Piso Antifatiga, Felpudo Vinilo con Logo, Felpudo Vinilo en Rollos). Las fotos no quedaron guardadas como archivo en este repo (se compartieron pegadas en el chat, no como adjunto).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>CAMBIOS EN ESTA VERSIÓN (v3)</t>
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>CAMBIOS EN ESTA VERSIÓN (v4)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>1. La marca y espesor de la base ahora se elige SIEMPRE (con o sin logo), no solo cuando no lleva logo. Se unificó una sola tabla de materiales en S//m², convirtiendo los precios de rollo (S//m lineal) a S//m² dividiendo entre el ancho fijo del rollo (1.20 m) — supuesto a validar: asume que cortar un ancho menor al del rollo completo cuesta proporcionalmente lo mismo por m².</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>2. Se agregó 'Complejidad del logo' (Simple ×0.8 / Media ×1.0 / Compleja ×1.2) como factor independiente del tamaño, que afecta SOLO el costo de material extra. Solo el nivel 'Media' está calibrado con datos reales (los 4 ejemplos manuscritos); Simple y Compleja son ESTIMACIONES (marcadas en ámbar en 'Datos Base', sección 1b) — deben ajustarse en cuanto haya ejemplos reales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>3. La mano de obra de 'Felpudo con Logo' YA NO se calcula con una fórmula (fijo + variable×área) — el usuario indicó que en la práctica paga 4 niveles fijos según tamaño y complejidad combinados: Nivel 1 = S/100, Nivel 2 = S/120, Nivel 3 = S/150, Nivel 4 = S/180 (Datos Base, sección 1c). El nivel se elige a mano en el Cotizador — no hay una regla automática que lo derive de ancho/alto, porque el usuario junta tamaño y complejidad en un solo criterio de su propio juicio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>2. División clara de responsabilidades (corregido por el usuario tras dos iteraciones): el COSTO DE MATERIAL EXTRA del logo depende SOLO del tamaño del felpudo (0.20m o 0.30m de ribete × S/94.90/m, tarifa Multilop 12mm de la foto original) — la complejidad NO lo toca. La MANO DE OBRA depende SOLO de la complejidad del logo, con 3 tarifas fijas: Simple = S/100, Media = S/120 (la única calibrada con un dato real: el ejemplo Vet. Orbegoso 1.20×0.90m), Compleja = S/150. Se eliminó el intento anterior de 4 'niveles' combinados y el multiplicador de complejidad sobre material — el usuario prefirió este modelo más simple de dos variables independientes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>CÓMO SE DERIVARON LAS FÓRMULAS ORIGINALES (nivel 'Media')</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Los valores base se obtuvieron por ingeniería inversa de los 4 (con logo) y 3 (mixtos) ejemplos manuscritos, ajustando una relación lineal (Costo = fijo + variable × área). El ajuste coincide casi exacto con los ejemplos de 'con logo' (diferencias de centavos por redondeo manual). En 'mixtos' el ajuste es un poco menos preciso (solo 3 puntos de datos).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="19" t="inlineStr">
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>OTROS SUPUESTOS A VALIDAR CON EL USUARIO</t>
         </is>
       </c>
     </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>3. Longitud extra (ribete) en 'con logo': se asumió 0.20 m para áreas menores a 1.00 m² y 0.30 m para el resto. No está confirmado si la regla real depende del área, del tamaño del logo, o de la complejidad — con más ejemplos se podría fusionar este concepto con el factor de complejidad.</t>
+        </is>
+      </c>
+    </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>3. Longitud extra (ribete) en 'con logo': se asumió 0.20 m para áreas menores a 1.00 m² y 0.30 m para el resto. No está confirmado si la regla real depende del área, del tamaño del logo, o de la complejidad — con más ejemplos se podría fusionar este concepto con el factor de complejidad.</t>
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>4. Ajuste fijo de acabado ('tapiz'): varía entre S/23 y S/25 en las notas originales. Se usó S/25 como estándar, sin ligarlo a la complejidad — confirmar si debería variar por complejidad también.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>4. Ajuste fijo de acabado ('tapiz'): varía entre S/23 y S/25 en las notas originales. Se usó S/25 como estándar, sin ligarlo a la complejidad — confirmar si debería variar por complejidad también.</t>
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>5. Paolo 15mm: en la sección de COSTOS de la foto 3 aparece como S/90.00, pero el cálculo de VENTA (S/158.00) solo cuadra si el costo es S/95.00. Se usó S/95.00 — confirmar cuál es correcto.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>5. Paolo 15mm: en la sección de COSTOS de la foto 3 aparece como S/90.00, pero el cálculo de VENTA (S/158.00) solo cuadra si el costo es S/95.00. Se usó S/95.00 — confirmar cuál es correcto.</t>
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>6. Mano de obra de 'Felpudos Mixtos': interpolada linealmente con solo 3 puntos de datos — es la fórmula menos confiable del archivo.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>6. Mano de obra de 'Felpudos Mixtos': interpolada linealmente con solo 3 puntos de datos — es la fórmula menos confiable del archivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>7. Piso Antifatiga: solo hay 1 ejemplo de precio por marca/espesor (a 1.50×0.90m) — no hay forma de confirmar si el costo por m² escala igual a otros tamaños.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="19" t="inlineStr">
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>CÓMO USAR EL COTIZADOR</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>En la pestaña 'Cotizador', llenar solo las celdas amarillas. El precio se recalcula solo. Si se actualiza algún costo real o se calibran los multiplicadores de complejidad, actualizarlo en 'Datos Base' y todo el cotizador se ajusta automáticamente.</t>
         </is>

</xml_diff>